<commit_message>
adicionado tratamentos  na tabela
</commit_message>
<xml_diff>
--- a/data/lancamentos.xlsx
+++ b/data/lancamentos.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -487,6 +487,32 @@
         </is>
       </c>
       <c r="F2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DESPESA</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>46100</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ESSENCIAIS</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>teste</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ajustes excel em drive
</commit_message>
<xml_diff>
--- a/data/lancamentos.xlsx
+++ b/data/lancamentos.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -474,25 +474,25 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ESSENCIAIS</t>
+          <t>VARIAVEIS</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>teste</t>
+          <t>PASSAGEM</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>16.93</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -500,20 +500,254 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
+        <v>46101</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>VARIAVEIS</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>JOGOS</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>61.93</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DESPESA</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>46101</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>VARIAVEIS</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>COMIDA</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DESPESA</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
         <v>46100</v>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>ESSENCIAIS</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>teste</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>RESERVA</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>RESERVA</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>140.4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DESPESA</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>46100</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>LAZER</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>RE3 REMAKE</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>140.4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DESPESA</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>46100</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>VARIAVEIS</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>RE3 REMAKE</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>11</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DESPESA</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>46100</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>VARIAVEIS</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>PASSAGEM</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>RECEITA</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>46100</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>VARIAVEIS</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>DINHEIRO PARA COMPRAR COMIDA</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>13</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DESPESA</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>46100</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>VARIAVEIS</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>COMIDA</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>94.34999999999999</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>14</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DESPESA</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>46100</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>VARIAVEIS</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>COMIDA</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>15</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DESPESA</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>46100</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>VARIAVEIS</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>COMIDA</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>16.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>